<commit_message>
uketsuke-stamp: anonymize department sheet names in fixture
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/uketsuke-stamp/tests/fixtures/sample-出欠表.xlsx
+++ b/uketsuke-stamp/tests/fixtures/sample-出欠表.xlsx
@@ -5,36 +5,36 @@
   <sheets>
     <sheet name="原本" sheetId="1" r:id="rId1"/>
     <sheet name="出欠合計表" sheetId="2" r:id="rId2"/>
-    <sheet name="01 役員" sheetId="3" r:id="rId3"/>
-    <sheet name="02 総務部" sheetId="4" r:id="rId4"/>
-    <sheet name="03 経理部" sheetId="5" r:id="rId5"/>
-    <sheet name="05 情報システム部" sheetId="6" r:id="rId6"/>
-    <sheet name="05 購買部" sheetId="7" r:id="rId7"/>
-    <sheet name="06 営業部" sheetId="8" r:id="rId8"/>
-    <sheet name="07 見積設計部" sheetId="9" r:id="rId9"/>
-    <sheet name="08 見積部" sheetId="10" r:id="rId10"/>
-    <sheet name="09 設計部" sheetId="11" r:id="rId11"/>
-    <sheet name="10 安全品質保証部" sheetId="12" r:id="rId12"/>
-    <sheet name="11 東京本店長" sheetId="13" r:id="rId13"/>
-    <sheet name="12 第一工事本部" sheetId="14" r:id="rId14"/>
-    <sheet name="13 栗島部" sheetId="15" r:id="rId15"/>
-    <sheet name="14 福田部" sheetId="16" r:id="rId16"/>
-    <sheet name="15 大通部" sheetId="17" r:id="rId17"/>
-    <sheet name="16 柳生部" sheetId="18" r:id="rId18"/>
-    <sheet name="17 第二工事本部" sheetId="19" r:id="rId19"/>
-    <sheet name="18 長靜部" sheetId="20" r:id="rId20"/>
-    <sheet name="19 富永部" sheetId="21" r:id="rId21"/>
-    <sheet name="20 前野部" sheetId="22" r:id="rId22"/>
-    <sheet name="21 加藤部" sheetId="23" r:id="rId23"/>
-    <sheet name="22 ＲＥ部" sheetId="24" r:id="rId24"/>
-    <sheet name="23 有賀部" sheetId="25" r:id="rId25"/>
-    <sheet name="24 工事管理部" sheetId="26" r:id="rId26"/>
-    <sheet name="25 直営課" sheetId="27" r:id="rId27"/>
-    <sheet name="26 ＣＡＤ課" sheetId="28" r:id="rId28"/>
-    <sheet name="27 横浜支店" sheetId="29" r:id="rId29"/>
-    <sheet name="28 東関東支店" sheetId="30" r:id="rId30"/>
-    <sheet name="29 北関東支店" sheetId="31" r:id="rId31"/>
-    <sheet name="３０ 大阪支店他" sheetId="32" r:id="rId32"/>
+    <sheet name="01 試験部01" sheetId="3" r:id="rId3"/>
+    <sheet name="02 試験部02" sheetId="4" r:id="rId4"/>
+    <sheet name="03 試験部03" sheetId="5" r:id="rId5"/>
+    <sheet name="05 試験部04" sheetId="6" r:id="rId6"/>
+    <sheet name="05 試験部05" sheetId="7" r:id="rId7"/>
+    <sheet name="06 試験部06" sheetId="8" r:id="rId8"/>
+    <sheet name="07 試験部07" sheetId="9" r:id="rId9"/>
+    <sheet name="08 試験部08" sheetId="10" r:id="rId10"/>
+    <sheet name="09 試験部09" sheetId="11" r:id="rId11"/>
+    <sheet name="10 試験部10" sheetId="12" r:id="rId12"/>
+    <sheet name="11 試験部11" sheetId="13" r:id="rId13"/>
+    <sheet name="12 試験部12" sheetId="14" r:id="rId14"/>
+    <sheet name="13 試験部13" sheetId="15" r:id="rId15"/>
+    <sheet name="14 試験部14" sheetId="16" r:id="rId16"/>
+    <sheet name="15 試験部15" sheetId="17" r:id="rId17"/>
+    <sheet name="16 試験部16" sheetId="18" r:id="rId18"/>
+    <sheet name="17 試験部17" sheetId="19" r:id="rId19"/>
+    <sheet name="18 試験部18" sheetId="20" r:id="rId20"/>
+    <sheet name="19 試験部19" sheetId="21" r:id="rId21"/>
+    <sheet name="20 試験部20" sheetId="22" r:id="rId22"/>
+    <sheet name="21 試験部21" sheetId="23" r:id="rId23"/>
+    <sheet name="22 試験部22" sheetId="24" r:id="rId24"/>
+    <sheet name="23 試験部23" sheetId="25" r:id="rId25"/>
+    <sheet name="24 試験部24" sheetId="26" r:id="rId26"/>
+    <sheet name="25 試験部25" sheetId="27" r:id="rId27"/>
+    <sheet name="26 試験部26" sheetId="28" r:id="rId28"/>
+    <sheet name="27 試験部27" sheetId="29" r:id="rId29"/>
+    <sheet name="28 試験部28" sheetId="30" r:id="rId30"/>
+    <sheet name="29 試験部29" sheetId="31" r:id="rId31"/>
+    <sheet name="３０ 試験部30" sheetId="32" r:id="rId32"/>
     <sheet name="Sheet2" sheetId="33" r:id="rId33"/>
     <sheet name="Sheet3" sheetId="34" r:id="rId34"/>
   </sheets>

</xml_diff>